<commit_message>
Small updates from Alex
</commit_message>
<xml_diff>
--- a/survey_results/EBS_results_metadata.xlsx
+++ b/survey_results/EBS_results_metadata.xlsx
@@ -1,23 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20416"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mike.levine\Work\github\KrillCommunication\survey_results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alex.derobertis\Work\Git-NOAA\KrillCommunication\survey_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18E2E791-AB46-4411-A662-E3EBA6067FCE}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="8070" activeTab="2" xr2:uid="{3F5CCE10-904A-496B-A773-B99F294FFA3C}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="21576" windowHeight="8076"/>
   </bookViews>
   <sheets>
     <sheet name="layer_results" sheetId="1" r:id="rId1"/>
     <sheet name="edsu_results" sheetId="2" r:id="rId2"/>
     <sheet name="survey_results" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -152,15 +151,6 @@
     <t xml:space="preserve">Krill nautical area scattering coefficient (m^2 nmi^-2) </t>
   </si>
   <si>
-    <t>Krill volumetric density (m^-3)</t>
-  </si>
-  <si>
-    <t>Krill areal density (m^-2)</t>
-  </si>
-  <si>
-    <t>Krill areal density in units of wet weight (g/m^-2)</t>
-  </si>
-  <si>
     <t>End time for the edsu (yyyy-mm-dd HH:MM:SS UTC)</t>
   </si>
   <si>
@@ -171,12 +161,21 @@
   </si>
   <si>
     <t>The total survey area (nmi^2)</t>
+  </si>
+  <si>
+    <t>Krill areal density (individuals m^-2)</t>
+  </si>
+  <si>
+    <t>Krill areal density in units of wet weight (g m^-2)</t>
+  </si>
+  <si>
+    <t>Krill volumetric density (individuals m^-3)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -521,15 +520,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72F96858-FA33-45E1-B8EF-DBC3C70F32F3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B23"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.5703125" customWidth="1"/>
-    <col min="2" max="2" width="11.7109375" customWidth="1"/>
+    <col min="1" max="1" width="24.5546875" customWidth="1"/>
+    <col min="2" max="2" width="11.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>21</v>
       </c>
@@ -537,7 +536,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -545,7 +544,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -553,7 +552,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -561,7 +560,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -569,7 +568,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -577,7 +576,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -585,7 +584,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -593,7 +592,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -601,15 +600,15 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B10" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -617,7 +616,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -625,7 +624,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>10</v>
       </c>
@@ -633,7 +632,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>11</v>
       </c>
@@ -641,7 +640,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>12</v>
       </c>
@@ -649,7 +648,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>13</v>
       </c>
@@ -657,7 +656,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>14</v>
       </c>
@@ -665,7 +664,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>15</v>
       </c>
@@ -673,7 +672,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>16</v>
       </c>
@@ -681,7 +680,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>17</v>
       </c>
@@ -689,28 +688,28 @@
         <v>40</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>18</v>
       </c>
       <c r="B21" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>19</v>
       </c>
       <c r="B22" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>20</v>
       </c>
       <c r="B23" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -719,14 +718,14 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7467A57-7D55-4223-9543-7B48A269F905}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="27.140625" customWidth="1"/>
+    <col min="1" max="1" width="27.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>21</v>
       </c>
@@ -734,7 +733,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -742,7 +741,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -750,7 +749,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -758,7 +757,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -766,7 +765,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -774,7 +773,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -782,7 +781,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -790,7 +789,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -798,15 +797,15 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B10" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -814,7 +813,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -822,7 +821,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -830,7 +829,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>10</v>
       </c>
@@ -838,7 +837,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>17</v>
       </c>
@@ -846,28 +845,28 @@
         <v>40</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>18</v>
       </c>
       <c r="B16" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>19</v>
       </c>
       <c r="B17" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>20</v>
       </c>
       <c r="B18" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -877,14 +876,14 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB622DFE-5E17-46DC-9AD7-EC0A487407C4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>21</v>
       </c>
@@ -892,7 +891,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -900,7 +899,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -908,15 +907,15 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B4" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -924,28 +923,28 @@
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>18</v>
       </c>
       <c r="B6" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>19</v>
       </c>
       <c r="B7" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>20</v>
       </c>
       <c r="B8" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
sharing PRELIMINARY 2004-2024 updated time series for exploratory analyses
</commit_message>
<xml_diff>
--- a/survey_results/EBS_results_metadata.xlsx
+++ b/survey_results/EBS_results_metadata.xlsx
@@ -1,20 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20416"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alex.derobertis\Work\Git-NOAA\KrillCommunication\survey_results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mike.levine\Work\github\KrillCommunication\survey_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7E16AD9-0CD0-4E32-9F22-A32F9E2F10E3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21576" windowHeight="8076"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="8070" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="layer_results" sheetId="1" r:id="rId1"/>
     <sheet name="edsu_results" sheetId="2" r:id="rId2"/>
     <sheet name="survey_results" sheetId="3" r:id="rId3"/>
+    <sheet name="survey issues and consideration" sheetId="6" r:id="rId4"/>
+    <sheet name="Lucca_2023_EBS_krill_120_kHz_TS" sheetId="4" r:id="rId5"/>
+    <sheet name="MACE_krill_catch_data" sheetId="5" r:id="rId6"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="73">
   <si>
     <t>ship</t>
   </si>
@@ -170,19 +174,158 @@
   </si>
   <si>
     <t>Krill volumetric density (individuals m^-3)</t>
+  </si>
+  <si>
+    <t>Region</t>
+  </si>
+  <si>
+    <t>length_mm</t>
+  </si>
+  <si>
+    <t>sigmaBS</t>
+  </si>
+  <si>
+    <t>TS</t>
+  </si>
+  <si>
+    <t>wet_wt_mg</t>
+  </si>
+  <si>
+    <t>column</t>
+  </si>
+  <si>
+    <t>krill length class (mm). Krill are lengthed from the curve of the carapace behind the eye to the posterior of the telson and placed in 1 mm bins.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Backscattering cross section (m^2) for a krill at length </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>l</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Target strength (dB re 1 m^2) for a krill at length </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>l</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Wet weight (mg) for a krill at length </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>l</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">The survey region that the TS-length table is developed for </t>
+  </si>
+  <si>
+    <t>haul</t>
+  </si>
+  <si>
+    <t>gear</t>
+  </si>
+  <si>
+    <t>length_bin</t>
+  </si>
+  <si>
+    <t>The event number that samples were collected from.</t>
+  </si>
+  <si>
+    <t>The gear used in the haul; generally Methot trawl gear</t>
+  </si>
+  <si>
+    <t>krill length measurement (mm). Krill are lengthed from the curve of the carapace behind the eye to the posterior of the telson.</t>
+  </si>
+  <si>
+    <t>The 1 mm length bin that the length_mm measurement was assigned to; this bin length is used to determine sigmaBS (see Lucca_2023_EBS_krill_120_kHz_TS tab)</t>
+  </si>
+  <si>
+    <t>Survey</t>
+  </si>
+  <si>
+    <t xml:space="preserve">various </t>
+  </si>
+  <si>
+    <t>issue</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">all years </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>≤ 2014</t>
+    </r>
+  </si>
+  <si>
+    <t>end position and time was not recorded for each edsu (only start positions and times are available)</t>
+  </si>
+  <si>
+    <t>data for this year should be considered PROVISIONAL as abundance was calculated using 2022 lengths. When 2024 length data are available, this year will be recalculated and the data set will be updated.</t>
+  </si>
+  <si>
+    <t>Survey was conducted with 3 Saildrone USVs as opposed to a research vessel. There was no biological data collection from the USVs, so krill lengths from 2018 are used to scale backscatter into abundance. These USVs only collected data to 200 m (as opposed to 500 m during vessel-based surveys). Based on other survey years, a mean of 4.3% of total observed krill backscatter was observed &gt; 200m. No correction is currently applied for this, although one was initially used. See Levine and De Robertis 2025 (https://doi.org/10.1016/j.fishres.2025.107270) for discussion.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -205,8 +348,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -520,15 +666,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B23"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.5546875" customWidth="1"/>
-    <col min="2" max="2" width="11.6640625" customWidth="1"/>
+    <col min="1" max="1" width="24.5703125" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>21</v>
       </c>
@@ -536,7 +682,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -544,7 +690,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -552,7 +698,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -560,7 +706,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -568,7 +714,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -576,7 +722,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -584,7 +730,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -592,7 +738,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -600,7 +746,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>42</v>
       </c>
@@ -608,7 +754,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -616,7 +762,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -624,7 +770,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>10</v>
       </c>
@@ -632,7 +778,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>11</v>
       </c>
@@ -640,7 +786,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>12</v>
       </c>
@@ -648,7 +794,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>13</v>
       </c>
@@ -656,7 +802,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>14</v>
       </c>
@@ -664,7 +810,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>15</v>
       </c>
@@ -672,7 +818,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>16</v>
       </c>
@@ -680,7 +826,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>17</v>
       </c>
@@ -688,7 +834,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>18</v>
       </c>
@@ -696,7 +842,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>19</v>
       </c>
@@ -704,7 +850,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>20</v>
       </c>
@@ -718,14 +864,14 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B18"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27.109375" customWidth="1"/>
+    <col min="1" max="1" width="27.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>21</v>
       </c>
@@ -733,7 +879,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -741,7 +887,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -749,7 +895,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -757,7 +903,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -765,7 +911,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -773,7 +919,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -781,7 +927,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -789,7 +935,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -797,7 +943,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>42</v>
       </c>
@@ -805,7 +951,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -813,7 +959,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -821,7 +967,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -829,7 +975,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>10</v>
       </c>
@@ -837,7 +983,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>17</v>
       </c>
@@ -845,7 +991,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>18</v>
       </c>
@@ -853,7 +999,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>19</v>
       </c>
@@ -861,7 +1007,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -876,14 +1022,14 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>21</v>
       </c>
@@ -891,7 +1037,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -899,7 +1045,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -907,7 +1053,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>43</v>
       </c>
@@ -915,7 +1061,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -923,7 +1069,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>18</v>
       </c>
@@ -931,7 +1077,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -939,7 +1085,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>20</v>
       </c>
@@ -951,4 +1097,193 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA08758F-21C2-4124-8FD8-3BFF89C37965}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="16.140625" customWidth="1"/>
+    <col min="3" max="3" width="90.28515625" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="94.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>202001</v>
+      </c>
+      <c r="B3">
+        <v>2020</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>202408</v>
+      </c>
+      <c r="B4">
+        <v>2024</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97156393-CD6C-41F6-AC67-93234F6A38F2}">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B5" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAD4D7A3-FAC6-48EB-85C8-93FF1EF1C1BA}">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B5" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>61</v>
+      </c>
+      <c r="B6" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fixed error- no length conversion was being applied to krill lengths used in Lucca 2021 TS model. Now lengths are converted to SL2 lengths.
</commit_message>
<xml_diff>
--- a/survey_results/EBS_results_metadata.xlsx
+++ b/survey_results/EBS_results_metadata.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mike.levine\Work\github\KrillCommunication\survey_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7E16AD9-0CD0-4E32-9F22-A32F9E2F10E3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DF83CF1-2FCD-464F-BF4D-CC528FE8029D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="8070" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="8070" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="layer_results" sheetId="1" r:id="rId1"/>
     <sheet name="edsu_results" sheetId="2" r:id="rId2"/>
     <sheet name="survey_results" sheetId="3" r:id="rId3"/>
     <sheet name="survey issues and consideration" sheetId="6" r:id="rId4"/>
-    <sheet name="Lucca_2023_EBS_krill_120_kHz_TS" sheetId="4" r:id="rId5"/>
+    <sheet name="Lucca_2021_EBS_krill_120_kHz_TS" sheetId="4" r:id="rId5"/>
     <sheet name="MACE_krill_catch_data" sheetId="5" r:id="rId6"/>
   </sheets>
   <calcPr calcId="162913"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="78">
   <si>
     <t>ship</t>
   </si>
@@ -192,9 +192,6 @@
   </si>
   <si>
     <t>column</t>
-  </si>
-  <si>
-    <t>krill length class (mm). Krill are lengthed from the curve of the carapace behind the eye to the posterior of the telson and placed in 1 mm bins.</t>
   </si>
   <si>
     <r>
@@ -299,6 +296,24 @@
   </si>
   <si>
     <t>Survey was conducted with 3 Saildrone USVs as opposed to a research vessel. There was no biological data collection from the USVs, so krill lengths from 2018 are used to scale backscatter into abundance. These USVs only collected data to 200 m (as opposed to 500 m during vessel-based surveys). Based on other survey years, a mean of 4.3% of total observed krill backscatter was observed &gt; 200m. No correction is currently applied for this, although one was initially used. See Levine and De Robertis 2025 (https://doi.org/10.1016/j.fishres.2025.107270) for discussion.</t>
+  </si>
+  <si>
+    <t>poland_length_mm</t>
+  </si>
+  <si>
+    <t>krill length class as measured at the Polish Sorting Center (mm). Krill are lengthed from the curve of the carapace behind the eye to the posterior of the telson and placed in 1 mm bins.</t>
+  </si>
+  <si>
+    <t>SL1_length_mm</t>
+  </si>
+  <si>
+    <t>Krill converted to 'Standard Length 1': anterior of the eye stalk to the posterior end of the telson and uropods. Conversion by Ressler 2012: 1.07 * poland_length_mm + 0.1041 (r2 = 0.96, n = 231)</t>
+  </si>
+  <si>
+    <t>SL2_length_mm</t>
+  </si>
+  <si>
+    <t>Krill converted to 'Standard Length 2' for use in Lucca 2021 TS modeling:  anterior of the eye to posterior of the sixth abdominal segment. Conversion by Lucca 2021: 0.82 * SL1_length_mm + -0.20 (r2 = 0.93, n = 273)</t>
   </si>
 </sst>
 </file>
@@ -1110,24 +1125,24 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B1" t="s">
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>69</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="94.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1138,7 +1153,7 @@
         <v>2020</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="45" x14ac:dyDescent="0.25">
@@ -1149,7 +1164,7 @@
         <v>2024</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -1159,10 +1174,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97156393-CD6C-41F6-AC67-93234F6A38F2}">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.85546875" customWidth="1"/>
+    <col min="1" max="1" width="20.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -1178,39 +1193,55 @@
         <v>48</v>
       </c>
       <c r="B2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>49</v>
+        <v>72</v>
       </c>
       <c r="B3" t="s">
-        <v>54</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>50</v>
+        <v>74</v>
       </c>
       <c r="B4" t="s">
-        <v>55</v>
+        <v>75</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>51</v>
+        <v>76</v>
       </c>
       <c r="B5" t="s">
-        <v>56</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B7" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>52</v>
       </c>
-      <c r="B6" t="s">
-        <v>57</v>
+      <c r="B8" t="s">
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -1245,18 +1276,18 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -1264,15 +1295,15 @@
         <v>49</v>
       </c>
       <c r="B5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
updated 2024 estimate using recently processed catch data from 2024 survey; added catch species composition data
</commit_message>
<xml_diff>
--- a/survey_results/EBS_results_metadata.xlsx
+++ b/survey_results/EBS_results_metadata.xlsx
@@ -1,24 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20416"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mike.levine\Work\github\KrillCommunication\survey_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DF83CF1-2FCD-464F-BF4D-CC528FE8029D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9C98F38-AF62-4870-B3DF-473CAB50E42D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="8070" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="8070" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="layer_results" sheetId="1" r:id="rId1"/>
     <sheet name="edsu_results" sheetId="2" r:id="rId2"/>
     <sheet name="survey_results" sheetId="3" r:id="rId3"/>
-    <sheet name="survey issues and consideration" sheetId="6" r:id="rId4"/>
-    <sheet name="Lucca_2021_EBS_krill_120_kHz_TS" sheetId="4" r:id="rId5"/>
-    <sheet name="MACE_krill_catch_data" sheetId="5" r:id="rId6"/>
+    <sheet name="Lucca_2021_EBS_krill_120_kHz_TS" sheetId="4" r:id="rId4"/>
+    <sheet name="MACE_krill_length_data" sheetId="5" r:id="rId5"/>
+    <sheet name="MACE_catch_species_comp_data" sheetId="7" r:id="rId6"/>
+    <sheet name="MACE_catch_locations" sheetId="8" r:id="rId7"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -30,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="94">
   <si>
     <t>ship</t>
   </si>
@@ -266,38 +267,6 @@
     <t>The 1 mm length bin that the length_mm measurement was assigned to; this bin length is used to determine sigmaBS (see Lucca_2023_EBS_krill_120_kHz_TS tab)</t>
   </si>
   <si>
-    <t>Survey</t>
-  </si>
-  <si>
-    <t xml:space="preserve">various </t>
-  </si>
-  <si>
-    <t>issue</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">all years </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>≤ 2014</t>
-    </r>
-  </si>
-  <si>
-    <t>end position and time was not recorded for each edsu (only start positions and times are available)</t>
-  </si>
-  <si>
-    <t>data for this year should be considered PROVISIONAL as abundance was calculated using 2022 lengths. When 2024 length data are available, this year will be recalculated and the data set will be updated.</t>
-  </si>
-  <si>
-    <t>Survey was conducted with 3 Saildrone USVs as opposed to a research vessel. There was no biological data collection from the USVs, so krill lengths from 2018 are used to scale backscatter into abundance. These USVs only collected data to 200 m (as opposed to 500 m during vessel-based surveys). Based on other survey years, a mean of 4.3% of total observed krill backscatter was observed &gt; 200m. No correction is currently applied for this, although one was initially used. See Levine and De Robertis 2025 (https://doi.org/10.1016/j.fishres.2025.107270) for discussion.</t>
-  </si>
-  <si>
     <t>poland_length_mm</t>
   </si>
   <si>
@@ -314,13 +283,82 @@
   </si>
   <si>
     <t>Krill converted to 'Standard Length 2' for use in Lucca 2021 TS modeling:  anterior of the eye to posterior of the sixth abdominal segment. Conversion by Lucca 2021: 0.82 * SL1_length_mm + -0.20 (r2 = 0.93, n = 273)</t>
+  </si>
+  <si>
+    <t>species_code</t>
+  </si>
+  <si>
+    <t>taxon</t>
+  </si>
+  <si>
+    <t>count</t>
+  </si>
+  <si>
+    <t>The species code used by the Polish Sorting center</t>
+  </si>
+  <si>
+    <t>Species or group name</t>
+  </si>
+  <si>
+    <t>Number of specimens counted within sample</t>
+  </si>
+  <si>
+    <t>SHIP</t>
+  </si>
+  <si>
+    <t>SURVEY</t>
+  </si>
+  <si>
+    <t>EVENT_ID</t>
+  </si>
+  <si>
+    <t>GEAR</t>
+  </si>
+  <si>
+    <t>EQ_TIME</t>
+  </si>
+  <si>
+    <t>EQ_LATITUDE</t>
+  </si>
+  <si>
+    <t>EQ_LONGITUDE</t>
+  </si>
+  <si>
+    <t>HEAD_ROPE_DEPTH</t>
+  </si>
+  <si>
+    <t>BOTTOM_DEPTH</t>
+  </si>
+  <si>
+    <t>HEAD_ROPE_TEMP</t>
+  </si>
+  <si>
+    <t>The ship code for the vessel conduting the survey. 21 = Miller Freeman; 157 = Oscar Dyson</t>
+  </si>
+  <si>
+    <t>Time and date (UTC) that the trawl reached depth and began fishing (EQ)</t>
+  </si>
+  <si>
+    <t>Longitude at the EQ point</t>
+  </si>
+  <si>
+    <t>Latitude at the EQ point</t>
+  </si>
+  <si>
+    <t>Average depth (m) of the top of Methot trawl during the trawl</t>
+  </si>
+  <si>
+    <t>Average bottom depth (m) along the trawl path</t>
+  </si>
+  <si>
+    <t>Average temperature (deg C) as recorded by a SBE temperature-depth probe attached to the trawl</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -335,12 +373,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -363,11 +395,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1115,64 +1144,6 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA08758F-21C2-4124-8FD8-3BFF89C37965}">
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="16.140625" customWidth="1"/>
-    <col min="3" max="3" width="90.28515625" style="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>65</v>
-      </c>
-      <c r="B1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>66</v>
-      </c>
-      <c r="B2" t="s">
-        <v>68</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="94.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>202001</v>
-      </c>
-      <c r="B3">
-        <v>2020</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>202408</v>
-      </c>
-      <c r="B4">
-        <v>2024</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>70</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97156393-CD6C-41F6-AC67-93234F6A38F2}">
   <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1198,26 +1169,26 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="B3" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="B4" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="B5" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -1250,14 +1221,75 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAD4D7A3-FAC6-48EB-85C8-93FF1EF1C1BA}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A2:B7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.85546875" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B5" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B6" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{702E8DCE-BC16-4514-A5E9-0BCAE72030BE}">
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>53</v>
@@ -1276,42 +1308,151 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>58</v>
+        <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>61</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="B5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="B6" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>2</v>
+        <v>72</v>
       </c>
       <c r="B7" t="s">
-        <v>25</v>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>73</v>
+      </c>
+      <c r="B8" t="s">
+        <v>76</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CCDF2FA-91AC-4813-B7FC-C27217CA4976}">
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B4" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>80</v>
+      </c>
+      <c r="B5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>81</v>
+      </c>
+      <c r="B6" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>82</v>
+      </c>
+      <c r="B7" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>83</v>
+      </c>
+      <c r="B8" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>84</v>
+      </c>
+      <c r="B9" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>85</v>
+      </c>
+      <c r="B10" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>86</v>
+      </c>
+      <c r="B11" t="s">
+        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
re-formatted krill catch and length data to be in per year files instead of a single combined file
</commit_message>
<xml_diff>
--- a/survey_results/EBS_results_metadata.xlsx
+++ b/survey_results/EBS_results_metadata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mike.levine\Work\github\KrillCommunication\survey_results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\github\KrillCommunication\survey_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9C98F38-AF62-4870-B3DF-473CAB50E42D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95B93BA9-025F-4D8A-97E5-122CB6A3DB87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="8070" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30360" yWindow="1560" windowWidth="21600" windowHeight="11295" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="layer_results" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="96">
   <si>
     <t>ship</t>
   </si>
@@ -352,6 +352,12 @@
   </si>
   <si>
     <t>Average temperature (deg C) as recorded by a SBE temperature-depth probe attached to the trawl</t>
+  </si>
+  <si>
+    <t>length_type</t>
+  </si>
+  <si>
+    <t>The method used to measure krill. 'poland' = standard laboratory processing at the Polish sorting center lab; 'scope' = at-sea microscope measurements; 'ai' = automated measurements using MACE ai/ml approach</t>
   </si>
 </sst>
 </file>
@@ -415,9 +421,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -455,7 +461,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -561,7 +567,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -703,7 +709,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1223,7 +1229,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAD4D7A3-FAC6-48EB-85C8-93FF1EF1C1BA}">
-  <dimension ref="A2:B7"/>
+  <dimension ref="A2:B8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.85546875" customWidth="1"/>
@@ -1239,42 +1245,50 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>58</v>
+        <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>61</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="B5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>60</v>
+        <v>94</v>
       </c>
       <c r="B6" t="s">
-        <v>64</v>
+        <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>2</v>
+        <v>49</v>
       </c>
       <c r="B7" t="s">
-        <v>25</v>
+        <v>63</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>60</v>
+      </c>
+      <c r="B8" t="s">
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -1361,7 +1375,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CCDF2FA-91AC-4813-B7FC-C27217CA4976}">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.85546875" customWidth="1"/>
@@ -1393,65 +1407,73 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>79</v>
+        <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>61</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B6" t="s">
-        <v>88</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B7" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B8" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B9" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B10" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>85</v>
+      </c>
+      <c r="B11" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>86</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B12" t="s">
         <v>93</v>
       </c>
     </row>

</xml_diff>